<commit_message>
docs(clase1): agregar presentacion del 05/08/2026 y actualizar lista de chequeo de requisitos
- Presentacion 'Clase 5 de Agosto 2026' (Calidad, Verificacion y Validacion, IEEE Std 1028-2008)
- Lista de chequeo de requisitos diligenciada para la revision entre pares del SRS
- README con objetivos y estructura del repositorio
</commit_message>
<xml_diff>
--- a/Clase#1/Tarea1/ListaChequeo_Requisitos_Software.xlsx
+++ b/Clase#1/Tarea1/ListaChequeo_Requisitos_Software.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andre\Documents\Semestre 9\Software 4\SRS TRABAJO OTRO EQUIPO\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andre\Documents\Semestre 9\Software 4\Trabajo\BITACORAS DE CLASE\Clase#1\Tarea1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1258BC2E-A5B8-4F5D-B4D3-1E4B248A44A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B4CA02A-3237-4BAB-8191-B6ECA57F5E4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard y Resumen" sheetId="1" r:id="rId1"/>

</xml_diff>